<commit_message>
Enhance GNSS functionality and error handling; update version and configuration settings
</commit_message>
<xml_diff>
--- a/lista hiriV_maleta.xlsx
+++ b/lista hiriV_maleta.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ale\Dropbox\clases_universidad\HIRI_PR0_FINAL_V01_ESTATIC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E667BBF-1BCC-4091-8EDE-E6C066C81B15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCF84DAE-D5F5-4A02-86E1-4E4086D846B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>NOMBRE</t>
   </si>
@@ -99,6 +99,9 @@
   </si>
   <si>
     <t>https://api-sensores.cmasccp.cl/insertarMedicion?idsSensores=1086,1087,1087,1088,1088,1088,1088,1088,1089,1090,1090,1090,1090,1090,1091,1092,1092&amp;idsVariables=53,54,55,11,12,15,45,46,4,3,6,7,8,9,51,3,6&amp;valores=Dioxido de Azufre (So2,ppm) ppm(1086),TVOC ppb(1087),eCO2 ppm(1087),Latitud °(1088),Longitud °(1088),Intensidad señal telefónica Adimensional(1088),Velocidad_km/h km/h(1088),Satelites int(1088),Voltaje V(1089),Grados celcius °C(1090),Humedad %(1090),Material particulado PM 1.0 µg/m³(1090),Material particulado PM 2.5 µg/m³(1090),Material particulado PM 10 µg/m³(1090),Material particulado PM 100 µg/m³(1091),Grados celcius °C(1092),Humedad %(1092)</t>
+  </si>
+  <si>
+    <t>https://api-sensores.cmasccp.cl/insertarMedicion?idsSensores=1100,1101,1101,1102,1102,1102,1102,1102,1103,1104,1104,1104,1104,1104,1105,1106,1106&amp;idsVariables=53,54,55,11,12,15,45,46,4,3,6,7,8,9,51,3,6&amp;valores=Dioxido de Azufre (So2,ppm) ppm(1100),TVOC ppb(1101),eCO2 ppm(1101),Latitud °(1102),Longitud °(1102),Intensidad señal telefónica Adimensional(1102),Velocidad_km/h km/h(1102),Satelites int(1102),Voltaje V(1103),Grados celcius °C(1104),Humedad %(1104),Material particulado PM 1.0 µg/m³(1104),Material particulado PM 2.5 µg/m³(1104),Material particulado PM 10 µg/m³(1104),Material particulado PM 100 µg/m³(1105),Grados celcius °C(1106),Humedad %(1106)</t>
   </si>
 </sst>
 </file>
@@ -546,12 +549,12 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="72.75">
+    <row r="9" spans="1:2" ht="105">
       <c r="A9" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>14</v>
+      <c r="B9" s="3" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="72.75">
@@ -574,6 +577,7 @@
   <hyperlinks>
     <hyperlink ref="B3" r:id="rId1" display="https://api-sensores.cmasccp.cl/insertarMedicion?idsSensores=1035,1036,1036,1037,1037,1037,1037,1037,1038,1039,1039,1039,1039,1039,1040,1041,1041&amp;idsVariables=53,54,55,11,12,15,45,46,4,3,6,7,8,9,51,3,6&amp;valores=Dioxido de Azufre (So2,ppm) ppm(1035),TVOC ppb(1036),eCO2 ppm(1036),Latitud °(1037),Longitud °(1037),Intensidad señal telefónica Adimensional(1037),Velocidad_km/h km/h(1037),Satelites int(1037),Voltaje V(1038),Grados celcius °C(1039),Humedad %(1039),Material particulado PM 1.0 µg/m³(1039),Material particulado PM 2.5 µg/m³(1039),Material particulado PM 10 µg/m³(1039),Material particulado PM 100 µg/m³(1040),Grados celcius °C(1041),Humedad %(1041)" xr:uid="{C866FE9F-AB0E-4BE8-9903-54F040F61F5D}"/>
     <hyperlink ref="B7" r:id="rId2" display="https://api-sensores.cmasccp.cl/insertarMedicion?idsSensores=1086,1087,1087,1088,1088,1088,1088,1088,1089,1090,1090,1090,1090,1090,1091,1092,1092&amp;idsVariables=53,54,55,11,12,15,45,46,4,3,6,7,8,9,51,3,6&amp;valores=Dioxido de Azufre (So2,ppm) ppm(1086),TVOC ppb(1087),eCO2 ppm(1087),Latitud °(1088),Longitud °(1088),Intensidad señal telefónica Adimensional(1088),Velocidad_km/h km/h(1088),Satelites int(1088),Voltaje V(1089),Grados celcius °C(1090),Humedad %(1090),Material particulado PM 1.0 µg/m³(1090),Material particulado PM 2.5 µg/m³(1090),Material particulado PM 10 µg/m³(1090),Material particulado PM 100 µg/m³(1091),Grados celcius °C(1092),Humedad %(1092)" xr:uid="{1A4416D1-AA41-4BF1-BCBD-7B1A08E768C9}"/>
+    <hyperlink ref="B9" r:id="rId3" display="https://api-sensores.cmasccp.cl/insertarMedicion?idsSensores=1100,1101,1101,1102,1102,1102,1102,1102,1103,1104,1104,1104,1104,1104,1105,1106,1106&amp;idsVariables=53,54,55,11,12,15,45,46,4,3,6,7,8,9,51,3,6&amp;valores=Dioxido de Azufre (So2,ppm) ppm(1100),TVOC ppb(1101),eCO2 ppm(1101),Latitud °(1102),Longitud °(1102),Intensidad señal telefónica Adimensional(1102),Velocidad_km/h km/h(1102),Satelites int(1102),Voltaje V(1103),Grados celcius °C(1104),Humedad %(1104),Material particulado PM 1.0 µg/m³(1104),Material particulado PM 2.5 µg/m³(1104),Material particulado PM 10 µg/m³(1104),Material particulado PM 100 µg/m³(1105),Grados celcius °C(1106),Humedad %(1106)" xr:uid="{E9EC897E-A763-4059-B2D8-05502F1E19AB}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>